<commit_message>
Refactor DRY, fix infinite Pager loop, update continuous playback behavior
</commit_message>
<xml_diff>
--- a/.agents/HOOKS_GUIDE.xlsx
+++ b/.agents/HOOKS_GUIDE.xlsx
@@ -9,22 +9,22 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص العام" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. خطاف البدء والافتتاح" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. خطاف النجاح والتحليل البع" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. خطاف الفحص والاختبار التل" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. خطاف معالجة الأخطاء والأع" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. خطاف مراجعة وتحديث المكتب" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. خطاف خط الإنتاج البرمجي" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. خطاف الإشراف العام وتصحيح" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. خطاف هندسة السياق" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. خطاف تدقيق الصيانة" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. خطاف التكامل الفني" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. خطاف الفحص الأمني" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. خطاف الذاكرة المستدامة" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. خطاف تنظيم وترتيب الأجهزة" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14. خطاف ترتيب الملفات لمسار " sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15. خطاف إدارة تليجرام" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16. خطاف إدارة النسخ والمستود" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17. خطاف تحديث الإنجازات" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. خطاف هندسة السياق" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. خطاف الإشراف العام وتصحيح" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. خطاف خط الإنتاج البرمجي" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. خطاف التكامل الفني" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. خطاف تدقيق الصيانة" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. خطاف الفحص الأمني" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. خطاف مراجعة وتحديث المكتب" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. خطاف الفحص والاختبار التل" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. خطاف معالجة الأخطاء والأع" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. خطاف إدارة النسخ والمستود" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. خطاف تحديث الإنجازات" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. خطاف الذاكرة المستدامة" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14. خطاف النجاح والتحليل البع" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15. خطاف تنظيم وترتيب الأجهزة" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16. خطاف ترتيب الملفات لمسار " sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17. خطاف إدارة تليجرام" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -560,37 +560,36 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2. خطاف النجاح والتحليل البعدي</t>
+          <t>2. خطاف هندسة السياق</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>تم بنجاح, انتهى المشروع بنجاح</t>
+          <t>سياق المشروع, هندسة السياق</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.1 Pro (High)`</t>
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[agent-optimizer]</t>
+          <t>[prompt-engineer], [agent-optimizer]</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
+          <t>إنشاء وتحديث ملف `PROJECT_CONTEXT.md` لضمان التوجيه وتفادي الانحراف التقني.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات التي واجهت الفريق والحلول البرمجية الفعالة التي تم تطبيقها.
-  2. **تحديث سجل التعلم (Learning Log):** توثيق المشاكل البرمجية المكتشفة وحلولها مباشرة في القسم الثامن من ملف `AGENTS.md` لتجنب تكرارها.
-  3. **تطوير مهارات الفريق:** مراجعة وتعديل مهارات الوكلاء وتحديث التعليمات تلقائياً.
-  4. **سد الفجوات البرمجية:** استدعاء الوكيل `[github-talent-scout]` للبحث عن أي مكتبات أو أدوات مفتوحة المصدر يمكنها تسريع العمل مستقبلاً ودمجها.</t>
+  1. **قراءة هيكل المشروع:** يقوم الوكيل `[prompt-engineer]` بتحليل البنية والقرارات المعمارية الحالية.
+  2. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` في مجلد المشروع ليعكس التحديثات المعمارية والقرارات التقنية.
+  3. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
         </is>
       </c>
     </row>
@@ -600,36 +599,36 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>3. خطاف الفحص والاختبار التلقائي</t>
+          <t>3. خطاف الإشراف العام وتصحيح المسار</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>قم بالاختبار, جاهز للتجربة</t>
+          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.1 Pro (High)`</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[android-testing], [code-reviewer-quality]</t>
+          <t>[prompt-engineer], [agent-optimizer]</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>تشغيل اختبارات الوحدة وفحص جودة الكود والأمان للتأكد من عدم وجود تراجعات.</t>
+          <t>تصحيح الخطافات الخاطئة والبرومبتات غير الاحترافية وتوجيهها للمسار الصحيح تلقائياً.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تشغيل الاختبارات:** تفعيل أدوات الفحص الآلي واختبارات الوحدة (Unit Tests).
-  2. **مراجعة الجودة:** التأكد من مطابقة الكود لمعايير النظافة والاتساق الهيكلي (Clean Code).
-  3. **تقرير الفحص:** تزويد المطور بتقرير واضح يوضح نجاح الاختبارات أو أي قصور يحتاج إلى تعديل.</t>
+  1. **الرصد التلقائي:** يقوم الوكيل الرئيسي بمراقبة المدخلات والبرومبتات. في حال تفعيل خطاف غير مناسب أو كتابة برومبت غير احترافي/مبهم، يتم اعتراض الطلب.
+  2. **استدعاء مهندس البرومبت (`prompt-engineer`):** يتدخل الوكيل تلقائياً لقراءة الطلب وإعادة صياغته وهندسته بطريقة احترافية تتوافق مع بيئة العمل.
+  3. **اختيار وتصحيح الخطاف:** يحدد الوكيل الفرعي `[prompt-engineer]` الخطاف المناسب الفعلي للطلب ويقوم بتحويل سياق العمل إليه تلقائياً لإكمال المهمة بدون مقاطعة المطور.</t>
         </is>
       </c>
     </row>
@@ -639,109 +638,31 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>4. خطاف معالجة الأخطاء والأعطال</t>
+          <t>4. خطاف خط الإنتاج البرمجي</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>حدث خطأ, التطبيق توقف, Crash</t>
+          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>[debugger]</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>* **طريقة العمل والإجراءات:**
-  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل.
-  2. **عزل المشكلة:** حصر الكود المسبب للأخطاء لمعرفة إن كان يتعلق بالشبكة، قاعدة البيانات، أو دورة حياة المكونات.
-  3. **اقتراح وتثبيت الحل:** تطبيق التعديل الأدنى الكافي لحل المشكلة مع حماية الأجزاء الأخرى من النظام.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>5. خطاف مراجعة وتحديث المكتبات</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>تحديث الاعتماديات, تحديث المكتبات</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>الأساسي: `Gemini 3.1 Pro (Low)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>[github-talent-scout], [code-architect]</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>فحص ملفات Gradle وتحديث المكتبات والاعتماديات القديمة وتجنب التعارضات.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الإصدارات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
-  2. **التحقق من التوافق:** دراسة التغييرات الجوهرية (Breaking Changes) في المكتبات المحدثة لضمان عدم كسر الكود الحالي.
-  3. **التحديث الآمن:** ترقية المكتبات تدريجياً واختبار البناء بعد كل ترقية.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>6. خطاف خط الإنتاج البرمجي</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.1 Pro (High)` 
  البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [android-testing]</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، المراجعة، الفحص والاختبار).</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **التصميم المعماري الهيكلي (`code-architect`):** يبدأ برسم معمارية الميزة وتحديد مواقع وتسمية الملفات الجديدة/المعدلة في الهيكل المناسب (Data/Domain/UI).
@@ -751,42 +672,120 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>5. خطاف التكامل الفني</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ربط API, تكامل خارجي</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>[devops-deployer], [backend-architect]</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
+  2. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.
+  3. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>6. خطاف تدقيق الصيانة</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>تدقيق صيانة, مراجعة DRY</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>[code-reviewer-quality], [performance-optimizer]</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **فحص الكود المكرر:** استدعاء الوكيل `[code-reviewer-quality]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY).
+  2. **فحص Recomposition:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
+  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود.</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7. خطاف الإشراف العام وتصحيح المسار</t>
+          <t>7. خطاف الفحص الأمني</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
+          <t>فحص أمني, مراجعة أمان</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.1 Pro (High)`</t>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[prompt-engineer], [agent-optimizer]</t>
+          <t>[security-auditor], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>تصحيح الخطافات الخاطئة والبرومبتات غير الاحترافية وتوجيهها للمسار الصحيح تلقائياً.</t>
+          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **الرصد التلقائي:** يقوم الوكيل الرئيسي بمراقبة المدخلات والبرومبتات. في حال تفعيل خطاف غير مناسب أو كتابة برومبت غير احترافي/مبهم، يتم اعتراض الطلب.
-  2. **استدعاء مهندس البرومبت (`prompt-engineer`):** يتدخل الوكيل تلقائياً لقراءة الطلب وإعادة صياغته وهندسته بطريقة احترافية تتوافق مع بيئة العمل.
-  3. **اختيار وتصحيح الخطاف:** يحدد الوكيل الفرعي `[prompt-engineer]` الخطاف المناسب الفعلي للطلب ويقوم بتحويل سياق العمل إليه تلقائياً لإكمال المهمة بدون مقاطعة المطور.</t>
+  1. **مسح الثغرات:** فحص الكود للتحقق من عدم وجود ثغرات OWASP الشائعة.
+  2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
+  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة والجلسات وحمايتها محلياً وسحابياً.</t>
         </is>
       </c>
     </row>
@@ -796,36 +795,36 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>8. خطاف هندسة السياق</t>
+          <t>8. خطاف مراجعة وتحديث المكتبات</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>سياق المشروع, هندسة السياق</t>
+          <t>تحديث الاعتماديات, تحديث المكتبات</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+          <t>الأساسي: `Gemini 3.1 Pro (Low)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[prompt-engineer], [agent-optimizer]</t>
+          <t>[github-talent-scout], [code-architect]</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>إنشاء وتحديث ملف `PROJECT_CONTEXT.md` لضمان التوجيه وتفادي الانحراف التقني.</t>
+          <t>فحص ملفات Gradle وتحديث المكتبات والاعتماديات القديمة وتجنب التعارضات.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة هيكل المشروع:** يقوم الوكيل `[prompt-engineer]` بتحليل البنية والقرارات المعمارية الحالية.
-  2. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` في مجلد المشروع ليعكس التحديثات المعمارية والقرارات التقنية.
-  3. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
+  1. **فحص الإصدارات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
+  2. **التحقق من التوافق:** دراسة التغييرات الجوهرية (Breaking Changes) في المكتبات المحدثة لضمان عدم كسر الكود الحالي.
+  3. **التحديث الآمن:** ترقية المكتبات تدريجياً واختبار البناء بعد كل ترقية.</t>
         </is>
       </c>
     </row>
@@ -835,12 +834,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>9. خطاف تدقيق الصيانة</t>
+          <t>9. خطاف الفحص والاختبار التلقائي</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>تدقيق صيانة, مراجعة DRY</t>
+          <t>قم بالاختبار, جاهز للتجربة</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -851,20 +850,20 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [performance-optimizer]</t>
+          <t>[android-testing], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية.</t>
+          <t>تشغيل اختبارات الوحدة وفحص جودة الكود والأمان للتأكد من عدم وجود تراجعات.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود المكرر:** استدعاء الوكيل `[code-reviewer-quality]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY).
-  2. **فحص Recomposition:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
-  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود.</t>
+  1. **تشغيل الاختبارات:** تفعيل أدوات الفحص الآلي واختبارات الوحدة (Unit Tests).
+  2. **مراجعة الجودة:** التأكد من مطابقة الكود لمعايير النظافة والاتساق الهيكلي (Clean Code).
+  3. **تقرير الفحص:** تزويد المطور بتقرير واضح يوضح نجاح الاختبارات أو أي قصور يحتاج إلى تعديل.</t>
         </is>
       </c>
     </row>
@@ -874,12 +873,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>10. خطاف التكامل الفني</t>
+          <t>10. خطاف معالجة الأخطاء والأعطال</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ربط API, تكامل خارجي</t>
+          <t>حدث خطأ, التطبيق توقف, Crash</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -890,20 +889,20 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[devops-deployer], [backend-architect]</t>
+          <t>[debugger]</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
+          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
-  2. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.
-  3. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
+  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل.
+  2. **عزل المشكلة:** حصر الكود المسبب للأخطاء لمعرفة إن كان يتعلق بالشبكة، قاعدة البيانات، أو دورة حياة المكونات.
+  3. **اقتراح وتثبيت الحل:** تطبيق التعديل الأدنى الكافي لحل المشكلة مع حماية الأجزاء الأخرى من النظام.</t>
         </is>
       </c>
     </row>
@@ -913,12 +912,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>11. خطاف الفحص الأمني</t>
+          <t>11. خطاف إدارة النسخ والمستودعات</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>فحص أمني, مراجعة أمان</t>
+          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -929,20 +928,20 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[security-auditor], [code-reviewer-quality]</t>
+          <t>[git-github-manager]</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
+          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مسح الثغرات:** فحص الكود للتحقق من عدم وجود ثغرات OWASP الشائعة.
-  2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
-  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة والجلسات وحمايتها محلياً وسحابياً.</t>
+  1. **التحقق من حالة المستودع:** فحص حالة Git باستخدام `git status` ومعرفة الملفات المعدلة والمحذوفة والجديدة.
+  2. **التنظيم والتصنيف:** مساعدة المطور في فرز الملفات، واستثناء الملفات غير الضرورية (تحديث `.gitignore`).
+  3. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وواضحة، وإنشاء فروع عند الحاجة (Branching)، وحل تعارضات الدمج، ثم دفع التغييرات إلى GitHub بأمان.</t>
         </is>
       </c>
     </row>
@@ -952,31 +951,70 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>12. خطاف الذاكرة المستدامة</t>
+          <t>12. خطاف تحديث الإنجازات</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>[git-github-manager]</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>صياغة التعديلات الأخيرة كإنجازات احترافية، كتابتها في README.md، ثم رفعها مباشرة إلى GitHub.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
+  2. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
+  3. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>13. خطاف الذاكرة المستدامة</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>حفظ ذاكرة, تحديث السياق, سجّل هذا</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
  البديل: `Gemini 3.1 Pro (High)`</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>[persistent-memory-engine]</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>التقاط الدروس والقرارات وتخزينها في MEMORY_STORE.md وتصديرها للوكلاء.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية واستخراج الدروس المستفادة، القرارات المعمارية، التفضيلات، والأخطاء المحلولة.
@@ -987,37 +1025,77 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>13. خطاف تنظيم وترتيب الأجهزة الشامل</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>14. خطاف النجاح والتحليل البعدي</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>تم بنجاح, انتهى المشروع بنجاح</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.1 Pro (High)`</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>[agent-optimizer]</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات التي واجهت الفريق والحلول البرمجية الفعالة التي تم تطبيقها.
+  2. **تحديث سجل التعلم (Learning Log):** توثيق المشاكل البرمجية المكتشفة وحلولها مباشرة في القسم الثامن من ملف `AGENTS.md` لتجنب تكرارها.
+  3. **تطوير مهارات الفريق:** مراجعة وتعديل مهارات الوكلاء وتحديث التعليمات تلقائياً.
+  4. **سد الفجوات البرمجية:** استدعاء الوكيل `[github-talent-scout]` للبحث عن أي مكتبات أو أدوات مفتوحة المصدر يمكنها تسريع العمل مستقبلاً ودمجها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>15. خطاف تنظيم وترتيب الأجهزة الشامل</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>رتب جهازى, فرز الملفات, ترتيب ملفات</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.1 Pro (High)` 
  البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>[windows-c-drive-optimizer], [windows-file-organizer]</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>ترتيب ملفات جذور الأقراص بالكامل مع تنظيف وتحسين مساحة قرص الـ C بآن واحد.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **فرز وتصنيف جذور الأقراص:** نقل الملفات السائبة بالكامل لمجلدات مخصصة وآمنة.
@@ -1026,37 +1104,37 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>14. خطاف ترتيب الملفات لمسار محدد</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>16. خطاف ترتيب الملفات لمسار محدد</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>رتب المسار, نظم المجلد, ترتيب مسار</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.6 Flash (Medium)` 
  البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>[windows-file-organizer]</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>تنظيم وفرز الملفات داخل مجلد أو مسار مخصص يحدده المستخدم بذكاء ودقة.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **تحديد وفحص المسار المستهدف:** التحقق من وجود المجلد المخصص وقراءة هيكل الملفات والمجلدات بداخله.
@@ -1065,121 +1143,43 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>15. خطاف إدارة تليجرام</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>17. خطاف إدارة تليجرام</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>شغل البوت, تفعيل تليجرام, Telegram Bot</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.6 Flash (Low)` 
  البديل: `Gemini 3.5 Flash (Low)`</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>[devops-deployer], [persistent-memory-engine]</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>تشغيل بوت تليجرام في الخلفية بنمط الاستماع للطلبات عن بعد دون تعارض.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **التحقق من البيئة:** فحص وجود رمز البوت (TELEGRAM_BOT_TOKEN) والاعتماديات.
   2. **معالجة التعارض (Conflict Resolution):** رصد وإنهاء أي عمليات بوت سابقة معلقة (معالجة خطأ 409 Conflict) عبر `taskkill`.
   3. **التشغيل بنمط الاستماع الفردي:** تشغيل السكربت `poll_once.py` في الخلفية (One-Shot Polling) ليستمع لطلب واحد ويخرج، مما يوقظ الوكيل للعمل.
   4. **إشعار الجاهزية:** تأكيد نجاح التشغيل واستعداد البوت لاستقبال الأوامر عبر التطبيق.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>16. خطاف إدارة النسخ والمستودعات</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>[git-github-manager]</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من حالة المستودع:** فحص حالة Git باستخدام `git status` ومعرفة الملفات المعدلة والمحذوفة والجديدة.
-  2. **التنظيم والتصنيف:** مساعدة المطور في فرز الملفات، واستثناء الملفات غير الضرورية (تحديث `.gitignore`).
-  3. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وواضحة، وإنشاء فروع عند الحاجة (Branching)، وحل تعارضات الدمج، ثم دفع التغييرات إلى GitHub بأمان.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>17. خطاف تحديث الإنجازات</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>[git-github-manager]</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>صياغة التعديلات الأخيرة كإنجازات احترافية، كتابتها في README.md، ثم رفعها مباشرة إلى GitHub.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
-  3. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>9. خطاف تدقيق الصيانة</t>
+          <t>9. خطاف الفحص والاختبار التلقائي</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تدقيق صيانة, مراجعة DRY</t>
+          <t>قم بالاختبار, جاهز للتجربة</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1265,20 +1265,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [performance-optimizer]</t>
+          <t>[android-testing], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية.</t>
+          <t>تشغيل اختبارات الوحدة وفحص جودة الكود والأمان للتأكد من عدم وجود تراجعات.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود المكرر:** استدعاء الوكيل `[code-reviewer-quality]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY).
-  2. **فحص Recomposition:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
-  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود.</t>
+  1. **تشغيل الاختبارات:** تفعيل أدوات الفحص الآلي واختبارات الوحدة (Unit Tests).
+  2. **مراجعة الجودة:** التأكد من مطابقة الكود لمعايير النظافة والاتساق الهيكلي (Clean Code).
+  3. **تقرير الفحص:** تزويد المطور بتقرير واضح يوضح نجاح الاختبارات أو أي قصور يحتاج إلى تعديل.</t>
         </is>
       </c>
     </row>
@@ -1348,12 +1348,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>10. خطاف التكامل الفني</t>
+          <t>10. خطاف معالجة الأخطاء والأعطال</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ربط API, تكامل خارجي</t>
+          <t>حدث خطأ, التطبيق توقف, Crash</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1364,20 +1364,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[devops-deployer], [backend-architect]</t>
+          <t>[debugger]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
+          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
-  2. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.
-  3. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
+  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل.
+  2. **عزل المشكلة:** حصر الكود المسبب للأخطاء لمعرفة إن كان يتعلق بالشبكة، قاعدة البيانات، أو دورة حياة المكونات.
+  3. **اقتراح وتثبيت الحل:** تطبيق التعديل الأدنى الكافي لحل المشكلة مع حماية الأجزاء الأخرى من النظام.</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>11. خطاف الفحص الأمني</t>
+          <t>11. خطاف إدارة النسخ والمستودعات</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>فحص أمني, مراجعة أمان</t>
+          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1463,20 +1463,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[security-auditor], [code-reviewer-quality]</t>
+          <t>[git-github-manager]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
+          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مسح الثغرات:** فحص الكود للتحقق من عدم وجود ثغرات OWASP الشائعة.
-  2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
-  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة والجلسات وحمايتها محلياً وسحابياً.</t>
+  1. **التحقق من حالة المستودع:** فحص حالة Git باستخدام `git status` ومعرفة الملفات المعدلة والمحذوفة والجديدة.
+  2. **التنظيم والتصنيف:** مساعدة المطور في فرز الملفات، واستثناء الملفات غير الضرورية (تحديث `.gitignore`).
+  3. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وواضحة، وإنشاء فروع عند الحاجة (Branching)، وحل تعارضات الدمج، ثم دفع التغييرات إلى GitHub بأمان.</t>
         </is>
       </c>
     </row>
@@ -1546,38 +1546,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>12. خطاف الذاكرة المستدامة</t>
+          <t>12. خطاف تحديث الإنجازات</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>حفظ ذاكرة, تحديث السياق, سجّل هذا</t>
+          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.1 Pro (High)`</t>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[persistent-memory-engine]</t>
+          <t>[git-github-manager]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>التقاط الدروس والقرارات وتخزينها في MEMORY_STORE.md وتصديرها للوكلاء.</t>
+          <t>صياغة التعديلات الأخيرة كإنجازات احترافية، كتابتها في README.md، ثم رفعها مباشرة إلى GitHub.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية واستخراج الدروس المستفادة، القرارات المعمارية، التفضيلات، والأخطاء المحلولة.
-  2. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
-  3. **الفهرسة (Index):** تصنيف كل ذاكرة حسب النوع (lesson/decision/preference/pattern/bug-fix/tool-discovery) ووسمها بأسماء الوكلاء المساهمين.
-  4. **التصدير الانتقائي (Export):** تحديث حزمة السياق لكل وكيل حسب بروتوكول التصدير في `MEMORY_EXPORT_PROTOCOL.md`.
-  5. **التنقيح (Prune):** مراجعة الذكريات القديمة وحذف المتقادمة أو المتناقضة.</t>
+  1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
+  2. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
+  3. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
         </is>
       </c>
     </row>
@@ -1647,36 +1645,38 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>13. خطاف تنظيم وترتيب الأجهزة الشامل</t>
+          <t>13. خطاف الذاكرة المستدامة</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>رتب جهازى, فرز الملفات, ترتيب ملفات</t>
+          <t>حفظ ذاكرة, تحديث السياق, سجّل هذا</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.1 Pro (High)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[windows-c-drive-optimizer], [windows-file-organizer]</t>
+          <t>[persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>ترتيب ملفات جذور الأقراص بالكامل مع تنظيف وتحسين مساحة قرص الـ C بآن واحد.</t>
+          <t>التقاط الدروس والقرارات وتخزينها في MEMORY_STORE.md وتصديرها للوكلاء.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فرز وتصنيف جذور الأقراص:** نقل الملفات السائبة بالكامل لمجلدات مخصصة وآمنة.
-  2. **تنظيف وتحسين النظام:** تحفيز وكيل C لضغط النظام وتفريغ الفيديوهات المؤقتة لزيادة السرعة والمساحة معاً.
-  3. **فحص سلامة الروابط وتوليد الفهارس:** التحقق من Junction Links وتحديث الفهارس لـ NotebookLM.</t>
+  1. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية واستخراج الدروس المستفادة، القرارات المعمارية، التفضيلات، والأخطاء المحلولة.
+  2. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
+  3. **الفهرسة (Index):** تصنيف كل ذاكرة حسب النوع (lesson/decision/preference/pattern/bug-fix/tool-discovery) ووسمها بأسماء الوكلاء المساهمين.
+  4. **التصدير الانتقائي (Export):** تحديث حزمة السياق لكل وكيل حسب بروتوكول التصدير في `MEMORY_EXPORT_PROTOCOL.md`.
+  5. **التنقيح (Prune):** مراجعة الذكريات القديمة وحذف المتقادمة أو المتناقضة.</t>
         </is>
       </c>
     </row>
@@ -1746,36 +1746,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>14. خطاف ترتيب الملفات لمسار محدد</t>
+          <t>14. خطاف النجاح والتحليل البعدي</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>رتب المسار, نظم المجلد, ترتيب مسار</t>
+          <t>تم بنجاح, انتهى المشروع بنجاح</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.6 Flash (Medium)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.1 Pro (High)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[windows-file-organizer]</t>
+          <t>[agent-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تنظيم وفرز الملفات داخل مجلد أو مسار مخصص يحدده المستخدم بذكاء ودقة.</t>
+          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تحديد وفحص المسار المستهدف:** التحقق من وجود المجلد المخصص وقراءة هيكل الملفات والمجلدات بداخله.
-  2. **تصنيف الملفات حسب النوع والتاريخ:** فرز الملفات حسب امتداداتها (مستندات، صور، فيديوهات، أكواد) أو تاريخ إنشائها.
-  3. **إعادة التسمية والتنظيم:** نقل الملفات إلى مجلدات فرعية مخصصة مع إعادة تسمية خالية من التعارضات.</t>
+  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات التي واجهت الفريق والحلول البرمجية الفعالة التي تم تطبيقها.
+  2. **تحديث سجل التعلم (Learning Log):** توثيق المشاكل البرمجية المكتشفة وحلولها مباشرة في القسم الثامن من ملف `AGENTS.md` لتجنب تكرارها.
+  3. **تطوير مهارات الفريق:** مراجعة وتعديل مهارات الوكلاء وتحديث التعليمات تلقائياً.
+  4. **سد الفجوات البرمجية:** استدعاء الوكيل `[github-talent-scout]` للبحث عن أي مكتبات أو أدوات مفتوحة المصدر يمكنها تسريع العمل مستقبلاً ودمجها.</t>
         </is>
       </c>
     </row>
@@ -1845,37 +1846,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>15. خطاف إدارة تليجرام</t>
+          <t>15. خطاف تنظيم وترتيب الأجهزة الشامل</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>شغل البوت, تفعيل تليجرام, Telegram Bot</t>
+          <t>رتب جهازى, فرز الملفات, ترتيب ملفات</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.6 Flash (Low)` 
- البديل: `Gemini 3.5 Flash (Low)`</t>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[devops-deployer], [persistent-memory-engine]</t>
+          <t>[windows-c-drive-optimizer], [windows-file-organizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تشغيل بوت تليجرام في الخلفية بنمط الاستماع للطلبات عن بعد دون تعارض.</t>
+          <t>ترتيب ملفات جذور الأقراص بالكامل مع تنظيف وتحسين مساحة قرص الـ C بآن واحد.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من البيئة:** فحص وجود رمز البوت (TELEGRAM_BOT_TOKEN) والاعتماديات.
-  2. **معالجة التعارض (Conflict Resolution):** رصد وإنهاء أي عمليات بوت سابقة معلقة (معالجة خطأ 409 Conflict) عبر `taskkill`.
-  3. **التشغيل بنمط الاستماع الفردي:** تشغيل السكربت `poll_once.py` في الخلفية (One-Shot Polling) ليستمع لطلب واحد ويخرج، مما يوقظ الوكيل للعمل.
-  4. **إشعار الجاهزية:** تأكيد نجاح التشغيل واستعداد البوت لاستقبال الأوامر عبر التطبيق.</t>
+  1. **فرز وتصنيف جذور الأقراص:** نقل الملفات السائبة بالكامل لمجلدات مخصصة وآمنة.
+  2. **تنظيف وتحسين النظام:** تحفيز وكيل C لضغط النظام وتفريغ الفيديوهات المؤقتة لزيادة السرعة والمساحة معاً.
+  3. **فحص سلامة الروابط وتوليد الفهارس:** التحقق من Junction Links وتحديث الفهارس لـ NotebookLM.</t>
         </is>
       </c>
     </row>
@@ -1945,36 +1945,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>16. خطاف إدارة النسخ والمستودعات</t>
+          <t>16. خطاف ترتيب الملفات لمسار محدد</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
+          <t>رتب المسار, نظم المجلد, ترتيب مسار</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+          <t>الأساسي: `Gemini 3.6 Flash (Medium)` 
  البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager]</t>
+          <t>[windows-file-organizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
+          <t>تنظيم وفرز الملفات داخل مجلد أو مسار مخصص يحدده المستخدم بذكاء ودقة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من حالة المستودع:** فحص حالة Git باستخدام `git status` ومعرفة الملفات المعدلة والمحذوفة والجديدة.
-  2. **التنظيم والتصنيف:** مساعدة المطور في فرز الملفات، واستثناء الملفات غير الضرورية (تحديث `.gitignore`).
-  3. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وواضحة، وإنشاء فروع عند الحاجة (Branching)، وحل تعارضات الدمج، ثم دفع التغييرات إلى GitHub بأمان.</t>
+  1. **تحديد وفحص المسار المستهدف:** التحقق من وجود المجلد المخصص وقراءة هيكل الملفات والمجلدات بداخله.
+  2. **تصنيف الملفات حسب النوع والتاريخ:** فرز الملفات حسب امتداداتها (مستندات، صور، فيديوهات، أكواد) أو تاريخ إنشائها.
+  3. **إعادة التسمية والتنظيم:** نقل الملفات إلى مجلدات فرعية مخصصة مع إعادة تسمية خالية من التعارضات.</t>
         </is>
       </c>
     </row>
@@ -2044,36 +2044,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>17. خطاف تحديث الإنجازات</t>
+          <t>17. خطاف إدارة تليجرام</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
+          <t>شغل البوت, تفعيل تليجرام, Telegram Bot</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+          <t>الأساسي: `Gemini 3.6 Flash (Low)` 
+ البديل: `Gemini 3.5 Flash (Low)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager]</t>
+          <t>[devops-deployer], [persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>صياغة التعديلات الأخيرة كإنجازات احترافية، كتابتها في README.md، ثم رفعها مباشرة إلى GitHub.</t>
+          <t>تشغيل بوت تليجرام في الخلفية بنمط الاستماع للطلبات عن بعد دون تعارض.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
-  3. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
+  1. **التحقق من البيئة:** فحص وجود رمز البوت (TELEGRAM_BOT_TOKEN) والاعتماديات.
+  2. **معالجة التعارض (Conflict Resolution):** رصد وإنهاء أي عمليات بوت سابقة معلقة (معالجة خطأ 409 Conflict) عبر `taskkill`.
+  3. **التشغيل بنمط الاستماع الفردي:** تشغيل السكربت `poll_once.py` في الخلفية (One-Shot Polling) ليستمع لطلب واحد ويخرج، مما يوقظ الوكيل للعمل.
+  4. **إشعار الجاهزية:** تأكيد نجاح التشغيل واستعداد البوت لاستقبال الأوامر عبر التطبيق.</t>
         </is>
       </c>
     </row>
@@ -2242,37 +2243,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2. خطاف النجاح والتحليل البعدي</t>
+          <t>2. خطاف هندسة السياق</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تم بنجاح, انتهى المشروع بنجاح</t>
+          <t>سياق المشروع, هندسة السياق</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.1 Pro (High)`</t>
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[agent-optimizer]</t>
+          <t>[prompt-engineer], [agent-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
+          <t>إنشاء وتحديث ملف `PROJECT_CONTEXT.md` لضمان التوجيه وتفادي الانحراف التقني.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات التي واجهت الفريق والحلول البرمجية الفعالة التي تم تطبيقها.
-  2. **تحديث سجل التعلم (Learning Log):** توثيق المشاكل البرمجية المكتشفة وحلولها مباشرة في القسم الثامن من ملف `AGENTS.md` لتجنب تكرارها.
-  3. **تطوير مهارات الفريق:** مراجعة وتعديل مهارات الوكلاء وتحديث التعليمات تلقائياً.
-  4. **سد الفجوات البرمجية:** استدعاء الوكيل `[github-talent-scout]` للبحث عن أي مكتبات أو أدوات مفتوحة المصدر يمكنها تسريع العمل مستقبلاً ودمجها.</t>
+  1. **قراءة هيكل المشروع:** يقوم الوكيل `[prompt-engineer]` بتحليل البنية والقرارات المعمارية الحالية.
+  2. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` في مجلد المشروع ليعكس التحديثات المعمارية والقرارات التقنية.
+  3. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
         </is>
       </c>
     </row>
@@ -2342,36 +2342,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>3. خطاف الفحص والاختبار التلقائي</t>
+          <t>3. خطاف الإشراف العام وتصحيح المسار</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>قم بالاختبار, جاهز للتجربة</t>
+          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.1 Pro (High)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[android-testing], [code-reviewer-quality]</t>
+          <t>[prompt-engineer], [agent-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تشغيل اختبارات الوحدة وفحص جودة الكود والأمان للتأكد من عدم وجود تراجعات.</t>
+          <t>تصحيح الخطافات الخاطئة والبرومبتات غير الاحترافية وتوجيهها للمسار الصحيح تلقائياً.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تشغيل الاختبارات:** تفعيل أدوات الفحص الآلي واختبارات الوحدة (Unit Tests).
-  2. **مراجعة الجودة:** التأكد من مطابقة الكود لمعايير النظافة والاتساق الهيكلي (Clean Code).
-  3. **تقرير الفحص:** تزويد المطور بتقرير واضح يوضح نجاح الاختبارات أو أي قصور يحتاج إلى تعديل.</t>
+  1. **الرصد التلقائي:** يقوم الوكيل الرئيسي بمراقبة المدخلات والبرومبتات. في حال تفعيل خطاف غير مناسب أو كتابة برومبت غير احترافي/مبهم، يتم اعتراض الطلب.
+  2. **استدعاء مهندس البرومبت (`prompt-engineer`):** يتدخل الوكيل تلقائياً لقراءة الطلب وإعادة صياغته وهندسته بطريقة احترافية تتوافق مع بيئة العمل.
+  3. **اختيار وتصحيح الخطاف:** يحدد الوكيل الفرعي `[prompt-engineer]` الخطاف المناسب الفعلي للطلب ويقوم بتحويل سياق العمل إليه تلقائياً لإكمال المهمة بدون مقاطعة المطور.</t>
         </is>
       </c>
     </row>
@@ -2441,36 +2441,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>4. خطاف معالجة الأخطاء والأعطال</t>
+          <t>4. خطاف خط الإنتاج البرمجي</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>حدث خطأ, التطبيق توقف, Crash</t>
+          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[debugger]</t>
+          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [android-testing]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
+          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، المراجعة، الفحص والاختبار).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل.
-  2. **عزل المشكلة:** حصر الكود المسبب للأخطاء لمعرفة إن كان يتعلق بالشبكة، قاعدة البيانات، أو دورة حياة المكونات.
-  3. **اقتراح وتثبيت الحل:** تطبيق التعديل الأدنى الكافي لحل المشكلة مع حماية الأجزاء الأخرى من النظام.</t>
+  1. **التصميم المعماري الهيكلي (`code-architect`):** يبدأ برسم معمارية الميزة وتحديد مواقع وتسمية الملفات الجديدة/المعدلة في الهيكل المناسب (Data/Domain/UI).
+  2. **الكتابة البرمجية والتطوير (`android-kotlin-pro` أو `jetpack-compose-ui`):** يتلقى التوجيهات المعمارية ويبدأ في تنفيذ الكود البرمجي وكتابة الواجهات طبقاً للملفات المحددة.
+  3. **المراجعة وضمان الجودة (`code-reviewer-quality`):** يفحص الكود بعد كتابته للتحقق من الاتساق، معالجة الاستثناءات، وخلوه من الثغرات الأمنية أو كود مهمل.
+  4. **الأتمتة والاختبار (`android-testing`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) لضمان ثبات الميزة المضافة وتغطيتها اختبارياً بالكامل قبل دمج الكود.</t>
         </is>
       </c>
     </row>
@@ -2540,36 +2541,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>5. خطاف مراجعة وتحديث المكتبات</t>
+          <t>5. خطاف التكامل الفني</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تحديث الاعتماديات, تحديث المكتبات</t>
+          <t>ربط API, تكامل خارجي</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.1 Pro (Low)` 
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
  البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[github-talent-scout], [code-architect]</t>
+          <t>[devops-deployer], [backend-architect]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>فحص ملفات Gradle وتحديث المكتبات والاعتماديات القديمة وتجنب التعارضات.</t>
+          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الإصدارات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
-  2. **التحقق من التوافق:** دراسة التغييرات الجوهرية (Breaking Changes) في المكتبات المحدثة لضمان عدم كسر الكود الحالي.
-  3. **التحديث الآمن:** ترقية المكتبات تدريجياً واختبار البناء بعد كل ترقية.</t>
+  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
+  2. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.
+  3. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
         </is>
       </c>
     </row>
@@ -2639,37 +2640,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>6. خطاف خط الإنتاج البرمجي</t>
+          <t>6. خطاف تدقيق الصيانة</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
+          <t>تدقيق صيانة, مراجعة DRY</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.1 Pro (High)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [android-testing]</t>
+          <t>[code-reviewer-quality], [performance-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، المراجعة، الفحص والاختبار).</t>
+          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التصميم المعماري الهيكلي (`code-architect`):** يبدأ برسم معمارية الميزة وتحديد مواقع وتسمية الملفات الجديدة/المعدلة في الهيكل المناسب (Data/Domain/UI).
-  2. **الكتابة البرمجية والتطوير (`android-kotlin-pro` أو `jetpack-compose-ui`):** يتلقى التوجيهات المعمارية ويبدأ في تنفيذ الكود البرمجي وكتابة الواجهات طبقاً للملفات المحددة.
-  3. **المراجعة وضمان الجودة (`code-reviewer-quality`):** يفحص الكود بعد كتابته للتحقق من الاتساق، معالجة الاستثناءات، وخلوه من الثغرات الأمنية أو كود مهمل.
-  4. **الأتمتة والاختبار (`android-testing`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) لضمان ثبات الميزة المضافة وتغطيتها اختبارياً بالكامل قبل دمج الكود.</t>
+  1. **فحص الكود المكرر:** استدعاء الوكيل `[code-reviewer-quality]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY).
+  2. **فحص Recomposition:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
+  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود.</t>
         </is>
       </c>
     </row>
@@ -2739,36 +2739,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>7. خطاف الإشراف العام وتصحيح المسار</t>
+          <t>7. خطاف الفحص الأمني</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
+          <t>فحص أمني, مراجعة أمان</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.1 Pro (High)`</t>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[prompt-engineer], [agent-optimizer]</t>
+          <t>[security-auditor], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تصحيح الخطافات الخاطئة والبرومبتات غير الاحترافية وتوجيهها للمسار الصحيح تلقائياً.</t>
+          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **الرصد التلقائي:** يقوم الوكيل الرئيسي بمراقبة المدخلات والبرومبتات. في حال تفعيل خطاف غير مناسب أو كتابة برومبت غير احترافي/مبهم، يتم اعتراض الطلب.
-  2. **استدعاء مهندس البرومبت (`prompt-engineer`):** يتدخل الوكيل تلقائياً لقراءة الطلب وإعادة صياغته وهندسته بطريقة احترافية تتوافق مع بيئة العمل.
-  3. **اختيار وتصحيح الخطاف:** يحدد الوكيل الفرعي `[prompt-engineer]` الخطاف المناسب الفعلي للطلب ويقوم بتحويل سياق العمل إليه تلقائياً لإكمال المهمة بدون مقاطعة المطور.</t>
+  1. **مسح الثغرات:** فحص الكود للتحقق من عدم وجود ثغرات OWASP الشائعة.
+  2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
+  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة والجلسات وحمايتها محلياً وسحابياً.</t>
         </is>
       </c>
     </row>
@@ -2838,36 +2838,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>8. خطاف هندسة السياق</t>
+          <t>8. خطاف مراجعة وتحديث المكتبات</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>سياق المشروع, هندسة السياق</t>
+          <t>تحديث الاعتماديات, تحديث المكتبات</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+          <t>الأساسي: `Gemini 3.1 Pro (Low)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[prompt-engineer], [agent-optimizer]</t>
+          <t>[github-talent-scout], [code-architect]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>إنشاء وتحديث ملف `PROJECT_CONTEXT.md` لضمان التوجيه وتفادي الانحراف التقني.</t>
+          <t>فحص ملفات Gradle وتحديث المكتبات والاعتماديات القديمة وتجنب التعارضات.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة هيكل المشروع:** يقوم الوكيل `[prompt-engineer]` بتحليل البنية والقرارات المعمارية الحالية.
-  2. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` في مجلد المشروع ليعكس التحديثات المعمارية والقرارات التقنية.
-  3. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
+  1. **فحص الإصدارات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
+  2. **التحقق من التوافق:** دراسة التغييرات الجوهرية (Breaking Changes) في المكتبات المحدثة لضمان عدم كسر الكود الحالي.
+  3. **التحديث الآمن:** ترقية المكتبات تدريجياً واختبار البناء بعد كل ترقية.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(hooks): integrate guard skills and add Hook 18 (Code Quality & Guard Audit Hook)
</commit_message>
<xml_diff>
--- a/.agents/HOOKS_GUIDE.xlsx
+++ b/.agents/HOOKS_GUIDE.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15. خطاف تنظيم وترتيب الأجهزة" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16. خطاف ترتيب الملفات لمسار " sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17. خطاف إدارة تليجرام" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18. خطاف التدقيق البرمجي الشا" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -587,9 +588,10 @@
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة هيكل المشروع:** يقوم الوكيل `[prompt-engineer]` بتحليل البنية والقرارات المعمارية الحالية.
-  2. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` في مجلد المشروع ليعكس التحديثات المعمارية والقرارات التقنية.
-  3. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
+  1. **مراجعة القواعد واستيراد الذاكرة العالمية:** يقوم الوكيل `[prompt-engineer]` بمراجعة الدستور المحلي والعالمي (`AGENTS.md`) بدقة، واستيراد البيانات من ملفات **الذاكرة العالمية (Global Memory)** و **الأنماط العالمية (Global Patterns)** لضمان تطبيق الدروس العابرة للمشاريع.
+  2. **قراءة هيكل المشروع:** تحليل البنية والقرارات المعمارية الحالية للمشروع.
+  3. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` ليعكس التحديثات المعمارية والقرارات التقنية.
+  4. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
         </is>
       </c>
     </row>
@@ -626,9 +628,10 @@
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **الرصد التلقائي:** يقوم الوكيل الرئيسي بمراقبة المدخلات والبرومبتات. في حال تفعيل خطاف غير مناسب أو كتابة برومبت غير احترافي/مبهم، يتم اعتراض الطلب.
-  2. **استدعاء مهندس البرومبت (`prompt-engineer`):** يتدخل الوكيل تلقائياً لقراءة الطلب وإعادة صياغته وهندسته بطريقة احترافية تتوافق مع بيئة العمل.
-  3. **اختيار وتصحيح الخطاف:** يحدد الوكيل الفرعي `[prompt-engineer]` الخطاف المناسب الفعلي للطلب ويقوم بتحويل سياق العمل إليه تلقائياً لإكمال المهمة بدون مقاطعة المطور.</t>
+  1. **الرصد التلقائي والإيقاف:** يقوم الوكيل الرئيسي بمراقبة المحادثة. عند استخدام المستخدم لمحفز "تصحيح مسار"، أو عند رصد دخول وكيل في دائرة مفرغة، يتم اعتراض العمل وإيقافه فوراً.
+  2. **التشريح الاستباقي الصارم (Prompt Autopsy &amp; Root-Cause Analysis):** يُمنع على `prompt-engineer` تقديم برومبت جديد مباشرة. يجب أولاً طباعة قسم `[ROOT-CAUSE ANALYSIS]` يشرح بوضوح سبب الانحراف السابق (هلوسة وكيل، غياب سياق، أو معمارية خاطئة).
+  3. **حماية السياق (Context Preservation):** تحديد المتطلبات أو الملفات التي كانت تنقص الوكيل السابق للعمل بشكل صحيح تحت قسم `[MISSING ARTIFACTS / INFO]`.
+  4. **إعادة الصياغة والتوجيه القاطع (Explicit Rerouting):** توليد التوجيه الهندسي الجديد تحت قسم `[RE-ENGINEERED PROMPT]` مقترناً بشكل صريح بالوكيل الفرعي المستهدف `[TARGET HOOK]` الذي سيستلم المهمة ليكملها بنظافة.</t>
         </is>
       </c>
     </row>
@@ -654,21 +657,23 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [android-testing]</t>
+          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [clean-code-guard], [android-testing], [test-guard]</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، المراجعة، الفحص والاختبار).</t>
+          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، حراسة الكود النظيف، والفحص والاختبار).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
+  0. **حقن السياق الإجباري (Mandatory Context Injection):** يُلزم الوكيل الرئيسي بتشغيل أداة حقن السياق (`python .agents/inject_context.py`) وتمرير مخرجاتها كـ `System Alert` أو `&gt; [!WARNING] Mandatory Constraints` في المحادثة قبل بدء أي عمل.
   1. **التصميم المعماري الهيكلي (`code-architect`):** يبدأ برسم معمارية الميزة وتحديد مواقع وتسمية الملفات الجديدة/المعدلة في الهيكل المناسب (Data/Domain/UI).
-  2. **الكتابة البرمجية والتطوير (`android-kotlin-pro` أو `jetpack-compose-ui`):** يتلقى التوجيهات المعمارية ويبدأ في تنفيذ الكود البرمجي وكتابة الواجهات طبقاً للملفات المحددة.
-  3. **المراجعة وضمان الجودة (`code-reviewer-quality`):** يفحص الكود بعد كتابته للتحقق من الاتساق، معالجة الاستثناءات، وخلوه من الثغرات الأمنية أو كود مهمل.
-  4. **الأتمتة والاختبار (`android-testing`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) لضمان ثبات الميزة المضافة وتغطيتها اختبارياً بالكامل قبل دمج الكود.</t>
+  2. **التدقيق المعماري الصارم وحلقة الـ 7 مرات (7-Iterations Devil's Advocate Loop):** يُمنع منعاً باتاً البدء بكتابة الكود. يجب إدخال خطة التنفيذ (`implementation_plan.md`) في حلقة مراجعة وتدقيق مع "محامي الشيطان" **لـ 7 مرات متتالية** حتى يتم سد كل الثغرات والوصول لنسبة نجاح 99.99% وتأمين قسم `[UNINTENDED SIDE-EFFECTS &amp; LIFECYCLE HAZARDS]` بالكامل قبل السماح بالكتابة.
+  3. **الكتابة البرمجية (Surgical Precision Execution):** يستلم الوكيل `[android-kotlin-pro]` أو `[jetpack-compose-ui]` الخطة المعتمدة ويبدأ بالتنفيذ. **يُحقن الوكيل بالبرومبت الإجباري التالي:** *(يُمنع منعاً باتاً المساس، أو تعديل، أو حذف أي كود حالي في المشروع لا ينص عليه صراحة في خطة التنفيذ. تصرف كجراح دقيق: أضف ميزتك فقط دون إحداث أي تغييرات جانبية في الملفات المفتوحة).*
+  4. **المراجعة وحراسة الكود النظيف (`code-reviewer-quality` + `clean-code-guard`):** يفحص الكود بعد كتابته للتحقق من الاتساق، وخلوه من أخطاء الـ AI الـ 14 الشائعة (ابتلاع الأخطاء، تضخم الدوال، الأكواد المكررة).
+  5. **الأتمتة والاختبار النظيف (`android-testing` + `test-guard`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) وفق معايير `test-guard` للتحقق من سلوك النظام الفعلي وليس فقط الـ Happy Path، وتجنب الـ Mocks المفرطة.</t>
         </is>
       </c>
     </row>
@@ -706,8 +711,9 @@
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
-  2. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.
-  3. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
+  2. **تحصين الانقطاع (API FAULT TOLERANCE CHECK):** يُمنع الدمج دون بناء `Interceptor` لمعالجة انقطاع الشبكة وإعادة المحاولة (Retry Mechanism)، وتغليف الردود بـ `Result&lt;T&gt;` أو `ErrorMapper` لمعالجة أخطاء HTTP (401, 404, 500).
+  3. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع وضمان التخزين المؤقت (Offline-First).
+  4. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
         </is>
       </c>
     </row>
@@ -722,7 +728,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>تدقيق صيانة, مراجعة DRY</t>
+          <t>تدقيق صيانة, مراجعة DRY, كود نظيف</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -733,20 +739,20 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [performance-optimizer]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [performance-optimizer]</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية.</t>
+          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية وتطبيق معايير الكود النظيف.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود المكرر:** استدعاء الوكيل `[code-reviewer-quality]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY).
-  2. **فحص Recomposition:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
-  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود.</t>
+  1. **فحص الكود النظيف والمكرر:** استدعاء الوكيل `[code-reviewer-quality]` و `[clean-code-guard]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY/KISS/YAGNI) والحد من التعقيد الحسابي.
+  2. **فحص Recomposition والأداء:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
+  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود وحذف الأكواد الميتة (Dead Code).</t>
         </is>
       </c>
     </row>
@@ -783,9 +789,9 @@
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مسح الثغرات:** فحص الكود للتحقق من عدم وجود ثغرات OWASP الشائعة.
+  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest للبحث عن المكونات المكشوفة (`Exported=true`)، وتسريب البيانات عبر `Intents` (Intent Hijacking)، وقواعد `ProGuard`.
   2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
-  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة والجلسات وحمايتها محلياً وسحابياً.</t>
+  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة و `SharedPreferences` والجلسات وحمايتها محلياً وسحابياً (إلزام إخراج تقرير يؤكد الفحص).</t>
         </is>
       </c>
     </row>
@@ -850,20 +856,21 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[android-testing], [code-reviewer-quality]</t>
+          <t>[android-testing], [test-guard], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>تشغيل اختبارات الوحدة وفحص جودة الكود والأمان للتأكد من عدم وجود تراجعات.</t>
+          <t>تشغيل اختبارات الوحدة وفحص جودة الكود واختبار السلوك الفعلي بدون Mock مفرط.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تشغيل الاختبارات:** تفعيل أدوات الفحص الآلي واختبارات الوحدة (Unit Tests).
-  2. **مراجعة الجودة:** التأكد من مطابقة الكود لمعايير النظافة والاتساق الهيكلي (Clean Code).
-  3. **تقرير الفحص:** تزويد المطور بتقرير واضح يوضح نجاح الاختبارات أو أي قصور يحتاج إلى تعديل.</t>
+  1. **التقمص (Persona):** يتصرف الوكيل كمدير فحص جودة صارم (Pre-Flight Inspector &amp; Senior DevOps QA). بصرامة تامة وبدون أي مجاملات.
+  2. **حراسة الاختبارات (`test-guard`):** التحقق من أن الاختبارات تفحص سلوك النظام الفعلي ومخرجاته القابلة للملاحظة، ومنع الاختبارات الوهمية (Tautological Tests) والـ Mocks الزائدة.
+  3. **قاعدة التغطية الإجبارية (TEST COVERAGE MANDATE):** يُرفض أي اختبار يغطي مسار النجاح فقط (Happy Path). يجب كتابة اختبار للنجاح، الفشل، والحالات الطرفية (مثل: Network Off، Configuration Change).
+  4. **تقرير الفحص الصارم:** تزويد المطور بتقرير يحاكي المطالبة القياسية: `[BLOCKERS]`, `[WARNINGS]`, `[PRE-FLIGHT FIXES]`, `[GO / NO-GO]`.</t>
         </is>
       </c>
     </row>
@@ -967,20 +974,21 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager]</t>
+          <t>[git-github-manager], [docs-guard]</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>صياغة التعديلات الأخيرة كإنجازات احترافية، كتابتها في README.md، ثم رفعها مباشرة إلى GitHub.</t>
+          <t>صياغة التعديلات كإنجازات ومطابقتها برمجياً عبر docs-guard ثم كتابتها في README.md ورفعها لـ GitHub.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
-  3. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
+  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs Drift).
+  3. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
+  4. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
         </is>
       </c>
     </row>
@@ -1017,9 +1025,9 @@
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية واستخراج الدروس المستفادة، القرارات المعمارية، التفضيلات، والأخطاء المحلولة.
-  2. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
-  3. **الفهرسة (Index):** تصنيف كل ذاكرة حسب النوع (lesson/decision/preference/pattern/bug-fix/tool-discovery) ووسمها بأسماء الوكلاء المساهمين.
+  1. **فلترة وتدقيق الدروس (LESSON VALIDATION):** يُمنع تسجيل معلومات بديهية أو عامة. يجب أن تكون الذكريات مركزة على القواعد المعمارية الجديدة، حيل تقنية فريدة، أو تحذيرات من أخطاء مكررة. يجب تضمين قسم `[ANTI-PATTERN AVOIDED]` لكل درس لمنع تكرار الخطأ.
+  2. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية لاستخراج القرارات المعمارية العميقة والحلول.
+  3. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
   4. **التصدير الانتقائي (Export):** تحديث حزمة السياق لكل وكيل حسب بروتوكول التصدير في `MEMORY_EXPORT_PROTOCOL.md`.
   5. **التنقيح (Prune):** مراجعة الذكريات القديمة وحذف المتقادمة أو المتناقضة.</t>
         </is>
@@ -1180,6 +1188,47 @@
   2. **معالجة التعارض (Conflict Resolution):** رصد وإنهاء أي عمليات بوت سابقة معلقة (معالجة خطأ 409 Conflict) عبر `taskkill`.
   3. **التشغيل بنمط الاستماع الفردي:** تشغيل السكربت `poll_once.py` في الخلفية (One-Shot Polling) ليستمع لطلب واحد ويخرج، مما يوقظ الوكيل للعمل.
   4. **إشعار الجاهزية:** تأكيد نجاح التشغيل واستعداد البوت لاستقبال الأوامر عبر التطبيق.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>18. خطاف التدقيق البرمجي الشامل وحراسة الجودة</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit, guard audit</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **فحص الكود النظيف (`clean-code-guard`):** مراجعة جميع التغييرات البرمجية الأخيرة للتأكد من عدم ابتلاع الأخطاء، صغر حجم الدوال، غياب الكود المكرر، ودقة التسميات ومطابقة المعايير المعمارية.
+  2. **حراسة جودة الاختبارات (`test-guard`):** فحص جميع ملفات الاختبار للتحقق من عدم وجود Mocks وهمية أو اختبارات فارغة لا تكتشف الأخطاء الحقيقية.
+  3. **حراسة التوثيق ومطابقة الرموز (`docs-guard`):** مطابقة كافة ملفات التوثيق والـ Markdown مع الكود البرمجي الفعلي لضمان عدم وجود أي انحراف (Docs-vs-Code Drift).
+  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.
+&lt;/div&gt;</t>
         </is>
       </c>
     </row>
@@ -1265,20 +1314,21 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[android-testing], [code-reviewer-quality]</t>
+          <t>[android-testing], [test-guard], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تشغيل اختبارات الوحدة وفحص جودة الكود والأمان للتأكد من عدم وجود تراجعات.</t>
+          <t>تشغيل اختبارات الوحدة وفحص جودة الكود واختبار السلوك الفعلي بدون Mock مفرط.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تشغيل الاختبارات:** تفعيل أدوات الفحص الآلي واختبارات الوحدة (Unit Tests).
-  2. **مراجعة الجودة:** التأكد من مطابقة الكود لمعايير النظافة والاتساق الهيكلي (Clean Code).
-  3. **تقرير الفحص:** تزويد المطور بتقرير واضح يوضح نجاح الاختبارات أو أي قصور يحتاج إلى تعديل.</t>
+  1. **التقمص (Persona):** يتصرف الوكيل كمدير فحص جودة صارم (Pre-Flight Inspector &amp; Senior DevOps QA). بصرامة تامة وبدون أي مجاملات.
+  2. **حراسة الاختبارات (`test-guard`):** التحقق من أن الاختبارات تفحص سلوك النظام الفعلي ومخرجاته القابلة للملاحظة، ومنع الاختبارات الوهمية (Tautological Tests) والـ Mocks الزائدة.
+  3. **قاعدة التغطية الإجبارية (TEST COVERAGE MANDATE):** يُرفض أي اختبار يغطي مسار النجاح فقط (Happy Path). يجب كتابة اختبار للنجاح، الفشل، والحالات الطرفية (مثل: Network Off، Configuration Change).
+  4. **تقرير الفحص الصارم:** تزويد المطور بتقرير يحاكي المطالبة القياسية: `[BLOCKERS]`, `[WARNINGS]`, `[PRE-FLIGHT FIXES]`, `[GO / NO-GO]`.</t>
         </is>
       </c>
     </row>
@@ -1562,20 +1612,21 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager]</t>
+          <t>[git-github-manager], [docs-guard]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>صياغة التعديلات الأخيرة كإنجازات احترافية، كتابتها في README.md، ثم رفعها مباشرة إلى GitHub.</t>
+          <t>صياغة التعديلات كإنجازات ومطابقتها برمجياً عبر docs-guard ثم كتابتها في README.md ورفعها لـ GitHub.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
-  3. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
+  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs Drift).
+  3. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
+  4. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
         </is>
       </c>
     </row>
@@ -1672,9 +1723,9 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية واستخراج الدروس المستفادة، القرارات المعمارية، التفضيلات، والأخطاء المحلولة.
-  2. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
-  3. **الفهرسة (Index):** تصنيف كل ذاكرة حسب النوع (lesson/decision/preference/pattern/bug-fix/tool-discovery) ووسمها بأسماء الوكلاء المساهمين.
+  1. **فلترة وتدقيق الدروس (LESSON VALIDATION):** يُمنع تسجيل معلومات بديهية أو عامة. يجب أن تكون الذكريات مركزة على القواعد المعمارية الجديدة، حيل تقنية فريدة، أو تحذيرات من أخطاء مكررة. يجب تضمين قسم `[ANTI-PATTERN AVOIDED]` لكل درس لمنع تكرار الخطأ.
+  2. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية لاستخراج القرارات المعمارية العميقة والحلول.
+  3. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
   4. **التصدير الانتقائي (Export):** تحديث حزمة السياق لكل وكيل حسب بروتوكول التصدير في `MEMORY_EXPORT_PROTOCOL.md`.
   5. **التنقيح (Prune):** مراجعة الذكريات القديمة وحذف المتقادمة أو المتناقضة.</t>
         </is>
@@ -2083,6 +2134,107 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>18. خطاف التدقيق البرمجي الشامل وحراسة الجودة</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit, guard audit</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Gemini 3.1 Pro (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **فحص الكود النظيف (`clean-code-guard`):** مراجعة جميع التغييرات البرمجية الأخيرة للتأكد من عدم ابتلاع الأخطاء، صغر حجم الدوال، غياب الكود المكرر، ودقة التسميات ومطابقة المعايير المعمارية.
+  2. **حراسة جودة الاختبارات (`test-guard`):** فحص جميع ملفات الاختبار للتحقق من عدم وجود Mocks وهمية أو اختبارات فارغة لا تكتشف الأخطاء الحقيقية.
+  3. **حراسة التوثيق ومطابقة الرموز (`docs-guard`):** مطابقة كافة ملفات التوثيق والـ Markdown مع الكود البرمجي الفعلي لضمان عدم وجود أي انحراف (Docs-vs-Code Drift).
+  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.
+&lt;/div&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2270,9 +2422,10 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة هيكل المشروع:** يقوم الوكيل `[prompt-engineer]` بتحليل البنية والقرارات المعمارية الحالية.
-  2. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` في مجلد المشروع ليعكس التحديثات المعمارية والقرارات التقنية.
-  3. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
+  1. **مراجعة القواعد واستيراد الذاكرة العالمية:** يقوم الوكيل `[prompt-engineer]` بمراجعة الدستور المحلي والعالمي (`AGENTS.md`) بدقة، واستيراد البيانات من ملفات **الذاكرة العالمية (Global Memory)** و **الأنماط العالمية (Global Patterns)** لضمان تطبيق الدروس العابرة للمشاريع.
+  2. **قراءة هيكل المشروع:** تحليل البنية والقرارات المعمارية الحالية للمشروع.
+  3. **توليد أو تحديث الملف:** كتابة أو تعديل ملف `PROJECT_CONTEXT.md` ليعكس التحديثات المعمارية والقرارات التقنية.
+  4. **التأكيد والمزامنة:** إعلام طاقم الوكلاء بالتحديثات المعتمدة لضمان التوافق.</t>
         </is>
       </c>
     </row>
@@ -2369,9 +2522,10 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **الرصد التلقائي:** يقوم الوكيل الرئيسي بمراقبة المدخلات والبرومبتات. في حال تفعيل خطاف غير مناسب أو كتابة برومبت غير احترافي/مبهم، يتم اعتراض الطلب.
-  2. **استدعاء مهندس البرومبت (`prompt-engineer`):** يتدخل الوكيل تلقائياً لقراءة الطلب وإعادة صياغته وهندسته بطريقة احترافية تتوافق مع بيئة العمل.
-  3. **اختيار وتصحيح الخطاف:** يحدد الوكيل الفرعي `[prompt-engineer]` الخطاف المناسب الفعلي للطلب ويقوم بتحويل سياق العمل إليه تلقائياً لإكمال المهمة بدون مقاطعة المطور.</t>
+  1. **الرصد التلقائي والإيقاف:** يقوم الوكيل الرئيسي بمراقبة المحادثة. عند استخدام المستخدم لمحفز "تصحيح مسار"، أو عند رصد دخول وكيل في دائرة مفرغة، يتم اعتراض العمل وإيقافه فوراً.
+  2. **التشريح الاستباقي الصارم (Prompt Autopsy &amp; Root-Cause Analysis):** يُمنع على `prompt-engineer` تقديم برومبت جديد مباشرة. يجب أولاً طباعة قسم `[ROOT-CAUSE ANALYSIS]` يشرح بوضوح سبب الانحراف السابق (هلوسة وكيل، غياب سياق، أو معمارية خاطئة).
+  3. **حماية السياق (Context Preservation):** تحديد المتطلبات أو الملفات التي كانت تنقص الوكيل السابق للعمل بشكل صحيح تحت قسم `[MISSING ARTIFACTS / INFO]`.
+  4. **إعادة الصياغة والتوجيه القاطع (Explicit Rerouting):** توليد التوجيه الهندسي الجديد تحت قسم `[RE-ENGINEERED PROMPT]` مقترناً بشكل صريح بالوكيل الفرعي المستهدف `[TARGET HOOK]` الذي سيستلم المهمة ليكملها بنظافة.</t>
         </is>
       </c>
     </row>
@@ -2457,21 +2611,23 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [android-testing]</t>
+          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [clean-code-guard], [android-testing], [test-guard]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، المراجعة، الفحص والاختبار).</t>
+          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، حراسة الكود النظيف، والفحص والاختبار).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
+  0. **حقن السياق الإجباري (Mandatory Context Injection):** يُلزم الوكيل الرئيسي بتشغيل أداة حقن السياق (`python .agents/inject_context.py`) وتمرير مخرجاتها كـ `System Alert` أو `&gt; [!WARNING] Mandatory Constraints` في المحادثة قبل بدء أي عمل.
   1. **التصميم المعماري الهيكلي (`code-architect`):** يبدأ برسم معمارية الميزة وتحديد مواقع وتسمية الملفات الجديدة/المعدلة في الهيكل المناسب (Data/Domain/UI).
-  2. **الكتابة البرمجية والتطوير (`android-kotlin-pro` أو `jetpack-compose-ui`):** يتلقى التوجيهات المعمارية ويبدأ في تنفيذ الكود البرمجي وكتابة الواجهات طبقاً للملفات المحددة.
-  3. **المراجعة وضمان الجودة (`code-reviewer-quality`):** يفحص الكود بعد كتابته للتحقق من الاتساق، معالجة الاستثناءات، وخلوه من الثغرات الأمنية أو كود مهمل.
-  4. **الأتمتة والاختبار (`android-testing`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) لضمان ثبات الميزة المضافة وتغطيتها اختبارياً بالكامل قبل دمج الكود.</t>
+  2. **التدقيق المعماري الصارم وحلقة الـ 7 مرات (7-Iterations Devil's Advocate Loop):** يُمنع منعاً باتاً البدء بكتابة الكود. يجب إدخال خطة التنفيذ (`implementation_plan.md`) في حلقة مراجعة وتدقيق مع "محامي الشيطان" **لـ 7 مرات متتالية** حتى يتم سد كل الثغرات والوصول لنسبة نجاح 99.99% وتأمين قسم `[UNINTENDED SIDE-EFFECTS &amp; LIFECYCLE HAZARDS]` بالكامل قبل السماح بالكتابة.
+  3. **الكتابة البرمجية (Surgical Precision Execution):** يستلم الوكيل `[android-kotlin-pro]` أو `[jetpack-compose-ui]` الخطة المعتمدة ويبدأ بالتنفيذ. **يُحقن الوكيل بالبرومبت الإجباري التالي:** *(يُمنع منعاً باتاً المساس، أو تعديل، أو حذف أي كود حالي في المشروع لا ينص عليه صراحة في خطة التنفيذ. تصرف كجراح دقيق: أضف ميزتك فقط دون إحداث أي تغييرات جانبية في الملفات المفتوحة).*
+  4. **المراجعة وحراسة الكود النظيف (`code-reviewer-quality` + `clean-code-guard`):** يفحص الكود بعد كتابته للتحقق من الاتساق، وخلوه من أخطاء الـ AI الـ 14 الشائعة (ابتلاع الأخطاء، تضخم الدوال، الأكواد المكررة).
+  5. **الأتمتة والاختبار النظيف (`android-testing` + `test-guard`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) وفق معايير `test-guard` للتحقق من سلوك النظام الفعلي وليس فقط الـ Happy Path، وتجنب الـ Mocks المفرطة.</t>
         </is>
       </c>
     </row>
@@ -2569,8 +2725,9 @@
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
-  2. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.
-  3. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
+  2. **تحصين الانقطاع (API FAULT TOLERANCE CHECK):** يُمنع الدمج دون بناء `Interceptor` لمعالجة انقطاع الشبكة وإعادة المحاولة (Retry Mechanism)، وتغليف الردود بـ `Result&lt;T&gt;` أو `ErrorMapper` لمعالجة أخطاء HTTP (401, 404, 500).
+  3. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع وضمان التخزين المؤقت (Offline-First).
+  4. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2802,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تدقيق صيانة, مراجعة DRY</t>
+          <t>تدقيق صيانة, مراجعة DRY, كود نظيف</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2656,20 +2813,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [performance-optimizer]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [performance-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية.</t>
+          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية وتطبيق معايير الكود النظيف.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود المكرر:** استدعاء الوكيل `[code-reviewer-quality]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY).
-  2. **فحص Recomposition:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
-  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود.</t>
+  1. **فحص الكود النظيف والمكرر:** استدعاء الوكيل `[code-reviewer-quality]` و `[clean-code-guard]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY/KISS/YAGNI) والحد من التعقيد الحسابي.
+  2. **فحص Recomposition والأداء:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
+  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود وحذف الأكواد الميتة (Dead Code).</t>
         </is>
       </c>
     </row>
@@ -2766,9 +2923,9 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مسح الثغرات:** فحص الكود للتحقق من عدم وجود ثغرات OWASP الشائعة.
+  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest للبحث عن المكونات المكشوفة (`Exported=true`)، وتسريب البيانات عبر `Intents` (Intent Hijacking)، وقواعد `ProGuard`.
   2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
-  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة والجلسات وحمايتها محلياً وسحابياً.</t>
+  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة و `SharedPreferences` والجلسات وحمايتها محلياً وسحابياً (إلزام إخراج تقرير يؤكد الفحص).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ecosystem): add resource-scout-integrator agent, Hook 19, and ecosystem sync script
</commit_message>
<xml_diff>
--- a/.agents/HOOKS_GUIDE.xlsx
+++ b/.agents/HOOKS_GUIDE.xlsx
@@ -26,6 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16. خطاف ترتيب الملفات لمسار " sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17. خطاف إدارة تليجرام" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18. خطاف التدقيق البرمجي الشا" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19. خطاف استكشاف وتكامل الموا" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -986,7 +987,7 @@
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs Drift).
+  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs-vs-Code Drift).
   3. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
   4. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
         </is>
@@ -1202,7 +1203,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit, guard audit</t>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1227,7 +1228,48 @@
   1. **فحص الكود النظيف (`clean-code-guard`):** مراجعة جميع التغييرات البرمجية الأخيرة للتأكد من عدم ابتلاع الأخطاء، صغر حجم الدوال، غياب الكود المكرر، ودقة التسميات ومطابقة المعايير المعمارية.
   2. **حراسة جودة الاختبارات (`test-guard`):** فحص جميع ملفات الاختبار للتحقق من عدم وجود Mocks وهمية أو اختبارات فارغة لا تكتشف الأخطاء الحقيقية.
   3. **حراسة التوثيق ومطابقة الرموز (`docs-guard`):** مطابقة كافة ملفات التوثيق والـ Markdown مع الكود البرمجي الفعلي لضمان عدم وجود أي انحراف (Docs-vs-Code Drift).
-  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.
+  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>19. خطاف استكشاف وتكامل الموارد العالمية</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.1 Pro (High)`</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [git-github-manager]</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها عالمياً وتحديث الخطافات ومزامنة مستودع Claude-Antigravity-Workspace.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **فحص وتقييم المورد (`resource-scout-integrator` + `github-talent-scout`):** استلام رابط المستودع الخارجي وفحص ملفات README والأكواد وتحديد ما إذا كان يُحدث نقلة نوعية واستبعاد ما لا يتوافق مع البيئة.
+  2. **بناء وهيكلة المهارات (`skill-forge-builder`):** استخراج المهارات الفعالة وصياغة ملفات `SKILL.md` وفق المعايير العالمية.
+  3. **التعميم العالمي (`global-deployment`):** نشر المهارات في `C:\Users\Kt\.gemini\config\skills/` لتصبح متاحة لكل المشاريع.
+  4. **تحديث الخطافات والإكسيل (`agent-optimizer`):** إضافة المهارات للخطافات ذات الصلة وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx`.
+  5. **مزامنة المستودع العام سحابياً (`git-github-manager`):** تشغيل `sync_global_ecosystem.py` لمزامنة كامل منظومة الوكلاء والمهارات والدليل مع مستودع `Claude-Antigravity-Workspace` ورفعه إلى GitHub.
 &lt;/div&gt;</t>
         </is>
       </c>
@@ -1624,7 +1666,7 @@
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs Drift).
+  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs-vs-Code Drift).
   3. **صياغة الإنجازات وتحديث README:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وإضافتها إلى ملف `README.md` الخاص بالمشروع.
   4. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديل على `README.md` وإجراء عملية الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
         </is>
@@ -2200,7 +2242,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit, guard audit</t>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2225,8 +2267,7 @@
   1. **فحص الكود النظيف (`clean-code-guard`):** مراجعة جميع التغييرات البرمجية الأخيرة للتأكد من عدم ابتلاع الأخطاء، صغر حجم الدوال، غياب الكود المكرر، ودقة التسميات ومطابقة المعايير المعمارية.
   2. **حراسة جودة الاختبارات (`test-guard`):** فحص جميع ملفات الاختبار للتحقق من عدم وجود Mocks وهمية أو اختبارات فارغة لا تكتشف الأخطاء الحقيقية.
   3. **حراسة التوثيق ومطابقة الرموز (`docs-guard`):** مطابقة كافة ملفات التوثيق والـ Markdown مع الكود البرمجي الفعلي لضمان عدم وجود أي انحراف (Docs-vs-Code Drift).
-  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.
-&lt;/div&gt;</t>
+  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.</t>
         </is>
       </c>
     </row>
@@ -2334,6 +2375,108 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>19. خطاف استكشاف وتكامل الموارد العالمية</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.1 Pro (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [git-github-manager]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها عالمياً وتحديث الخطافات ومزامنة مستودع Claude-Antigravity-Workspace.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **فحص وتقييم المورد (`resource-scout-integrator` + `github-talent-scout`):** استلام رابط المستودع الخارجي وفحص ملفات README والأكواد وتحديد ما إذا كان يُحدث نقلة نوعية واستبعاد ما لا يتوافق مع البيئة.
+  2. **بناء وهيكلة المهارات (`skill-forge-builder`):** استخراج المهارات الفعالة وصياغة ملفات `SKILL.md` وفق المعايير العالمية.
+  3. **التعميم العالمي (`global-deployment`):** نشر المهارات في `C:\Users\Kt\.gemini\config\skills/` لتصبح متاحة لكل المشاريع.
+  4. **تحديث الخطافات والإكسيل (`agent-optimizer`):** إضافة المهارات للخطافات ذات الصلة وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx`.
+  5. **مزامنة المستودع العام سحابياً (`git-github-manager`):** تشغيل `sync_global_ecosystem.py` لمزامنة كامل منظومة الوكلاء والمهارات والدليل مع مستودع `Claude-Antigravity-Workspace` ورفعه إلى GitHub.
+&lt;/div&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(prompt-library): update HOOKS_GUIDE, update_html, and sync script
</commit_message>
<xml_diff>
--- a/.agents/HOOKS_GUIDE.xlsx
+++ b/.agents/HOOKS_GUIDE.xlsx
@@ -1254,12 +1254,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [git-github-manager]</t>
+          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها عالمياً وتحديث الخطافات ومزامنة مستودع Claude-Antigravity-Workspace.</t>
+          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ومزامنة المنظومة.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1268,7 +1268,7 @@
   1. **فحص وتقييم المورد (`resource-scout-integrator` + `github-talent-scout`):** استلام رابط المستودع الخارجي وفحص ملفات README والأكواد وتحديد ما إذا كان يُحدث نقلة نوعية واستبعاد ما لا يتوافق مع البيئة.
   2. **بناء وهيكلة المهارات (`skill-forge-builder`):** استخراج المهارات الفعالة وصياغة ملفات `SKILL.md` وفق المعايير العالمية.
   3. **التعميم العالمي (`global-deployment`):** نشر المهارات في `C:\Users\Kt\.gemini\config\skills/` لتصبح متاحة لكل المشاريع.
-  4. **تحديث الخطافات والإكسيل (`agent-optimizer`):** إضافة المهارات للخطافات ذات الصلة وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx`.
+  4. **تحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر (`agent-optimizer` + `frontend-design-builder`):** إضافة المهارات للخطافات ذات الصلة وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx` وتشغيل `update_html.py` لتحديث تطبيق مكتبة الأوامر التفاعلي (`03_Dynamic_Prompt_Library/index.html`).
   5. **مزامنة المستودع العام سحابياً (`git-github-manager`):** تشغيل `sync_global_ecosystem.py` لمزامنة كامل منظومة الوكلاء والمهارات والدليل مع مستودع `Claude-Antigravity-Workspace` ورفعه إلى GitHub.
 &lt;/div&gt;</t>
         </is>
@@ -2452,12 +2452,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [git-github-manager]</t>
+          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها عالمياً وتحديث الخطافات ومزامنة مستودع Claude-Antigravity-Workspace.</t>
+          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ومزامنة المنظومة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
   1. **فحص وتقييم المورد (`resource-scout-integrator` + `github-talent-scout`):** استلام رابط المستودع الخارجي وفحص ملفات README والأكواد وتحديد ما إذا كان يُحدث نقلة نوعية واستبعاد ما لا يتوافق مع البيئة.
   2. **بناء وهيكلة المهارات (`skill-forge-builder`):** استخراج المهارات الفعالة وصياغة ملفات `SKILL.md` وفق المعايير العالمية.
   3. **التعميم العالمي (`global-deployment`):** نشر المهارات في `C:\Users\Kt\.gemini\config\skills/` لتصبح متاحة لكل المشاريع.
-  4. **تحديث الخطافات والإكسيل (`agent-optimizer`):** إضافة المهارات للخطافات ذات الصلة وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx`.
+  4. **تحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر (`agent-optimizer` + `frontend-design-builder`):** إضافة المهارات للخطافات ذات الصلة وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx` وتشغيل `update_html.py` لتحديث تطبيق مكتبة الأوامر التفاعلي (`03_Dynamic_Prompt_Library/index.html`).
   5. **مزامنة المستودع العام سحابياً (`git-github-manager`):** تشغيل `sync_global_ecosystem.py` لمزامنة كامل منظومة الوكلاء والمهارات والدليل مع مستودع `Claude-Antigravity-Workspace` ورفعه إلى GitHub.
 &lt;/div&gt;</t>
         </is>

</xml_diff>